<commit_message>
feat: add optional email anđ validate in email form
</commit_message>
<xml_diff>
--- a/public/templates/khach-moi.xlsx
+++ b/public/templates/khach-moi.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khách mời" sheetId="1" r:id="R6a5a24269fb34998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khách mời" sheetId="1" r:id="R1e1bef65debe4d87"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -282,6 +282,7 @@
     <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="47" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -309,6 +310,9 @@
       <x:c r="H1" s="4" t="str">
         <x:v>Ghi chú</x:v>
       </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Email</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -333,6 +337,7 @@
       <x:c r="H2" s="5" t="str">
         <x:v>Gia đình có hai trẻ nhỏ cần ghế</x:v>
       </x:c>
+      <x:c r="I2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="5" t="str">
@@ -357,6 +362,7 @@
       <x:c r="H3" s="5" t="str">
         <x:v>Muốn ngồi gần lối ra</x:v>
       </x:c>
+      <x:c r="I3" s="6"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="5" t="str">
@@ -381,6 +387,7 @@
       <x:c r="H4" s="5" t="str">
         <x:v>Đi cùng một người</x:v>
       </x:c>
+      <x:c r="I4" s="6"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="5" t="str">
@@ -403,6 +410,7 @@
       </x:c>
       <x:c r="G5" s="6" t="str"/>
       <x:c r="H5" s="5" t="str"/>
+      <x:c r="I5" s="6"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="str">
@@ -425,1491 +433,1987 @@
       </x:c>
       <x:c r="G6" s="6" t="str"/>
       <x:c r="H6" s="5" t="str"/>
+      <x:c r="I6" s="6"/>
     </x:row>
     <x:row r="7">
       <x:c r="G7" s="7"/>
+      <x:c r="I7" s="7"/>
     </x:row>
     <x:row r="8">
       <x:c r="G8" s="7"/>
+      <x:c r="I8" s="7"/>
     </x:row>
     <x:row r="9">
       <x:c r="G9" s="7"/>
+      <x:c r="I9" s="7"/>
     </x:row>
     <x:row r="10">
       <x:c r="G10" s="7"/>
+      <x:c r="I10" s="7"/>
     </x:row>
     <x:row r="11">
       <x:c r="G11" s="7"/>
+      <x:c r="I11" s="7"/>
     </x:row>
     <x:row r="12">
       <x:c r="G12" s="7"/>
+      <x:c r="I12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="G13" s="7"/>
+      <x:c r="I13" s="7"/>
     </x:row>
     <x:row r="14">
       <x:c r="G14" s="7"/>
+      <x:c r="I14" s="7"/>
     </x:row>
     <x:row r="15">
       <x:c r="G15" s="7"/>
+      <x:c r="I15" s="7"/>
     </x:row>
     <x:row r="16">
       <x:c r="G16" s="7"/>
+      <x:c r="I16" s="7"/>
     </x:row>
     <x:row r="17">
       <x:c r="G17" s="7"/>
+      <x:c r="I17" s="7"/>
     </x:row>
     <x:row r="18">
       <x:c r="G18" s="7"/>
+      <x:c r="I18" s="7"/>
     </x:row>
     <x:row r="19">
       <x:c r="G19" s="7"/>
+      <x:c r="I19" s="7"/>
     </x:row>
     <x:row r="20">
       <x:c r="G20" s="7"/>
+      <x:c r="I20" s="7"/>
     </x:row>
     <x:row r="21">
       <x:c r="G21" s="7"/>
+      <x:c r="I21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="G22" s="7"/>
+      <x:c r="I22" s="7"/>
     </x:row>
     <x:row r="23">
       <x:c r="G23" s="7"/>
+      <x:c r="I23" s="7"/>
     </x:row>
     <x:row r="24">
       <x:c r="G24" s="7"/>
+      <x:c r="I24" s="7"/>
     </x:row>
     <x:row r="25">
       <x:c r="G25" s="7"/>
+      <x:c r="I25" s="7"/>
     </x:row>
     <x:row r="26">
       <x:c r="G26" s="7"/>
+      <x:c r="I26" s="7"/>
     </x:row>
     <x:row r="27">
       <x:c r="G27" s="7"/>
+      <x:c r="I27" s="7"/>
     </x:row>
     <x:row r="28">
       <x:c r="G28" s="7"/>
+      <x:c r="I28" s="7"/>
     </x:row>
     <x:row r="29">
       <x:c r="G29" s="7"/>
+      <x:c r="I29" s="7"/>
     </x:row>
     <x:row r="30">
       <x:c r="G30" s="7"/>
+      <x:c r="I30" s="7"/>
     </x:row>
     <x:row r="31">
       <x:c r="G31" s="7"/>
+      <x:c r="I31" s="7"/>
     </x:row>
     <x:row r="32">
       <x:c r="G32" s="7"/>
+      <x:c r="I32" s="7"/>
     </x:row>
     <x:row r="33">
       <x:c r="G33" s="7"/>
+      <x:c r="I33" s="7"/>
     </x:row>
     <x:row r="34">
       <x:c r="G34" s="7"/>
+      <x:c r="I34" s="7"/>
     </x:row>
     <x:row r="35">
       <x:c r="G35" s="7"/>
+      <x:c r="I35" s="7"/>
     </x:row>
     <x:row r="36">
       <x:c r="G36" s="7"/>
+      <x:c r="I36" s="7"/>
     </x:row>
     <x:row r="37">
       <x:c r="G37" s="7"/>
+      <x:c r="I37" s="7"/>
     </x:row>
     <x:row r="38">
       <x:c r="G38" s="7"/>
+      <x:c r="I38" s="7"/>
     </x:row>
     <x:row r="39">
       <x:c r="G39" s="7"/>
+      <x:c r="I39" s="7"/>
     </x:row>
     <x:row r="40">
       <x:c r="G40" s="7"/>
+      <x:c r="I40" s="7"/>
     </x:row>
     <x:row r="41">
       <x:c r="G41" s="7"/>
+      <x:c r="I41" s="7"/>
     </x:row>
     <x:row r="42">
       <x:c r="G42" s="7"/>
+      <x:c r="I42" s="7"/>
     </x:row>
     <x:row r="43">
       <x:c r="G43" s="7"/>
+      <x:c r="I43" s="7"/>
     </x:row>
     <x:row r="44">
       <x:c r="G44" s="7"/>
+      <x:c r="I44" s="7"/>
     </x:row>
     <x:row r="45">
       <x:c r="G45" s="7"/>
+      <x:c r="I45" s="7"/>
     </x:row>
     <x:row r="46">
       <x:c r="G46" s="7"/>
+      <x:c r="I46" s="7"/>
     </x:row>
     <x:row r="47">
       <x:c r="G47" s="7"/>
+      <x:c r="I47" s="7"/>
     </x:row>
     <x:row r="48">
       <x:c r="G48" s="7"/>
+      <x:c r="I48" s="7"/>
     </x:row>
     <x:row r="49">
       <x:c r="G49" s="7"/>
+      <x:c r="I49" s="7"/>
     </x:row>
     <x:row r="50">
       <x:c r="G50" s="7"/>
+      <x:c r="I50" s="7"/>
     </x:row>
     <x:row r="51">
       <x:c r="G51" s="7"/>
+      <x:c r="I51" s="7"/>
     </x:row>
     <x:row r="52">
       <x:c r="G52" s="7"/>
+      <x:c r="I52" s="7"/>
     </x:row>
     <x:row r="53">
       <x:c r="G53" s="7"/>
+      <x:c r="I53" s="7"/>
     </x:row>
     <x:row r="54">
       <x:c r="G54" s="7"/>
+      <x:c r="I54" s="7"/>
     </x:row>
     <x:row r="55">
       <x:c r="G55" s="7"/>
+      <x:c r="I55" s="7"/>
     </x:row>
     <x:row r="56">
       <x:c r="G56" s="7"/>
+      <x:c r="I56" s="7"/>
     </x:row>
     <x:row r="57">
       <x:c r="G57" s="7"/>
+      <x:c r="I57" s="7"/>
     </x:row>
     <x:row r="58">
       <x:c r="G58" s="7"/>
+      <x:c r="I58" s="7"/>
     </x:row>
     <x:row r="59">
       <x:c r="G59" s="7"/>
+      <x:c r="I59" s="7"/>
     </x:row>
     <x:row r="60">
       <x:c r="G60" s="7"/>
+      <x:c r="I60" s="7"/>
     </x:row>
     <x:row r="61">
       <x:c r="G61" s="7"/>
+      <x:c r="I61" s="7"/>
     </x:row>
     <x:row r="62">
       <x:c r="G62" s="7"/>
+      <x:c r="I62" s="7"/>
     </x:row>
     <x:row r="63">
       <x:c r="G63" s="7"/>
+      <x:c r="I63" s="7"/>
     </x:row>
     <x:row r="64">
       <x:c r="G64" s="7"/>
+      <x:c r="I64" s="7"/>
     </x:row>
     <x:row r="65">
       <x:c r="G65" s="7"/>
+      <x:c r="I65" s="7"/>
     </x:row>
     <x:row r="66">
       <x:c r="G66" s="7"/>
+      <x:c r="I66" s="7"/>
     </x:row>
     <x:row r="67">
       <x:c r="G67" s="7"/>
+      <x:c r="I67" s="7"/>
     </x:row>
     <x:row r="68">
       <x:c r="G68" s="7"/>
+      <x:c r="I68" s="7"/>
     </x:row>
     <x:row r="69">
       <x:c r="G69" s="7"/>
+      <x:c r="I69" s="7"/>
     </x:row>
     <x:row r="70">
       <x:c r="G70" s="7"/>
+      <x:c r="I70" s="7"/>
     </x:row>
     <x:row r="71">
       <x:c r="G71" s="7"/>
+      <x:c r="I71" s="7"/>
     </x:row>
     <x:row r="72">
       <x:c r="G72" s="7"/>
+      <x:c r="I72" s="7"/>
     </x:row>
     <x:row r="73">
       <x:c r="G73" s="7"/>
+      <x:c r="I73" s="7"/>
     </x:row>
     <x:row r="74">
       <x:c r="G74" s="7"/>
+      <x:c r="I74" s="7"/>
     </x:row>
     <x:row r="75">
       <x:c r="G75" s="7"/>
+      <x:c r="I75" s="7"/>
     </x:row>
     <x:row r="76">
       <x:c r="G76" s="7"/>
+      <x:c r="I76" s="7"/>
     </x:row>
     <x:row r="77">
       <x:c r="G77" s="7"/>
+      <x:c r="I77" s="7"/>
     </x:row>
     <x:row r="78">
       <x:c r="G78" s="7"/>
+      <x:c r="I78" s="7"/>
     </x:row>
     <x:row r="79">
       <x:c r="G79" s="7"/>
+      <x:c r="I79" s="7"/>
     </x:row>
     <x:row r="80">
       <x:c r="G80" s="7"/>
+      <x:c r="I80" s="7"/>
     </x:row>
     <x:row r="81">
       <x:c r="G81" s="7"/>
+      <x:c r="I81" s="7"/>
     </x:row>
     <x:row r="82">
       <x:c r="G82" s="7"/>
+      <x:c r="I82" s="7"/>
     </x:row>
     <x:row r="83">
       <x:c r="G83" s="7"/>
+      <x:c r="I83" s="7"/>
     </x:row>
     <x:row r="84">
       <x:c r="G84" s="7"/>
+      <x:c r="I84" s="7"/>
     </x:row>
     <x:row r="85">
       <x:c r="G85" s="7"/>
+      <x:c r="I85" s="7"/>
     </x:row>
     <x:row r="86">
       <x:c r="G86" s="7"/>
+      <x:c r="I86" s="7"/>
     </x:row>
     <x:row r="87">
       <x:c r="G87" s="7"/>
+      <x:c r="I87" s="7"/>
     </x:row>
     <x:row r="88">
       <x:c r="G88" s="7"/>
+      <x:c r="I88" s="7"/>
     </x:row>
     <x:row r="89">
       <x:c r="G89" s="7"/>
+      <x:c r="I89" s="7"/>
     </x:row>
     <x:row r="90">
       <x:c r="G90" s="7"/>
+      <x:c r="I90" s="7"/>
     </x:row>
     <x:row r="91">
       <x:c r="G91" s="7"/>
+      <x:c r="I91" s="7"/>
     </x:row>
     <x:row r="92">
       <x:c r="G92" s="7"/>
+      <x:c r="I92" s="7"/>
     </x:row>
     <x:row r="93">
       <x:c r="G93" s="7"/>
+      <x:c r="I93" s="7"/>
     </x:row>
     <x:row r="94">
       <x:c r="G94" s="7"/>
+      <x:c r="I94" s="7"/>
     </x:row>
     <x:row r="95">
       <x:c r="G95" s="7"/>
+      <x:c r="I95" s="7"/>
     </x:row>
     <x:row r="96">
       <x:c r="G96" s="7"/>
+      <x:c r="I96" s="7"/>
     </x:row>
     <x:row r="97">
       <x:c r="G97" s="7"/>
+      <x:c r="I97" s="7"/>
     </x:row>
     <x:row r="98">
       <x:c r="G98" s="7"/>
+      <x:c r="I98" s="7"/>
     </x:row>
     <x:row r="99">
       <x:c r="G99" s="7"/>
+      <x:c r="I99" s="7"/>
     </x:row>
     <x:row r="100">
       <x:c r="G100" s="7"/>
+      <x:c r="I100" s="7"/>
     </x:row>
     <x:row r="101">
       <x:c r="G101" s="7"/>
+      <x:c r="I101" s="7"/>
     </x:row>
     <x:row r="102">
       <x:c r="G102" s="7"/>
+      <x:c r="I102" s="7"/>
     </x:row>
     <x:row r="103">
       <x:c r="G103" s="7"/>
+      <x:c r="I103" s="7"/>
     </x:row>
     <x:row r="104">
       <x:c r="G104" s="7"/>
+      <x:c r="I104" s="7"/>
     </x:row>
     <x:row r="105">
       <x:c r="G105" s="7"/>
+      <x:c r="I105" s="7"/>
     </x:row>
     <x:row r="106">
       <x:c r="G106" s="7"/>
+      <x:c r="I106" s="7"/>
     </x:row>
     <x:row r="107">
       <x:c r="G107" s="7"/>
+      <x:c r="I107" s="7"/>
     </x:row>
     <x:row r="108">
       <x:c r="G108" s="7"/>
+      <x:c r="I108" s="7"/>
     </x:row>
     <x:row r="109">
       <x:c r="G109" s="7"/>
+      <x:c r="I109" s="7"/>
     </x:row>
     <x:row r="110">
       <x:c r="G110" s="7"/>
+      <x:c r="I110" s="7"/>
     </x:row>
     <x:row r="111">
       <x:c r="G111" s="7"/>
+      <x:c r="I111" s="7"/>
     </x:row>
     <x:row r="112">
       <x:c r="G112" s="7"/>
+      <x:c r="I112" s="7"/>
     </x:row>
     <x:row r="113">
       <x:c r="G113" s="7"/>
+      <x:c r="I113" s="7"/>
     </x:row>
     <x:row r="114">
       <x:c r="G114" s="7"/>
+      <x:c r="I114" s="7"/>
     </x:row>
     <x:row r="115">
       <x:c r="G115" s="7"/>
+      <x:c r="I115" s="7"/>
     </x:row>
     <x:row r="116">
       <x:c r="G116" s="7"/>
+      <x:c r="I116" s="7"/>
     </x:row>
     <x:row r="117">
       <x:c r="G117" s="7"/>
+      <x:c r="I117" s="7"/>
     </x:row>
     <x:row r="118">
       <x:c r="G118" s="7"/>
+      <x:c r="I118" s="7"/>
     </x:row>
     <x:row r="119">
       <x:c r="G119" s="7"/>
+      <x:c r="I119" s="7"/>
     </x:row>
     <x:row r="120">
       <x:c r="G120" s="7"/>
+      <x:c r="I120" s="7"/>
     </x:row>
     <x:row r="121">
       <x:c r="G121" s="7"/>
+      <x:c r="I121" s="7"/>
     </x:row>
     <x:row r="122">
       <x:c r="G122" s="7"/>
+      <x:c r="I122" s="7"/>
     </x:row>
     <x:row r="123">
       <x:c r="G123" s="7"/>
+      <x:c r="I123" s="7"/>
     </x:row>
     <x:row r="124">
       <x:c r="G124" s="7"/>
+      <x:c r="I124" s="7"/>
     </x:row>
     <x:row r="125">
       <x:c r="G125" s="7"/>
+      <x:c r="I125" s="7"/>
     </x:row>
     <x:row r="126">
       <x:c r="G126" s="7"/>
+      <x:c r="I126" s="7"/>
     </x:row>
     <x:row r="127">
       <x:c r="G127" s="7"/>
+      <x:c r="I127" s="7"/>
     </x:row>
     <x:row r="128">
       <x:c r="G128" s="7"/>
+      <x:c r="I128" s="7"/>
     </x:row>
     <x:row r="129">
       <x:c r="G129" s="7"/>
+      <x:c r="I129" s="7"/>
     </x:row>
     <x:row r="130">
       <x:c r="G130" s="7"/>
+      <x:c r="I130" s="7"/>
     </x:row>
     <x:row r="131">
       <x:c r="G131" s="7"/>
+      <x:c r="I131" s="7"/>
     </x:row>
     <x:row r="132">
       <x:c r="G132" s="7"/>
+      <x:c r="I132" s="7"/>
     </x:row>
     <x:row r="133">
       <x:c r="G133" s="7"/>
+      <x:c r="I133" s="7"/>
     </x:row>
     <x:row r="134">
       <x:c r="G134" s="7"/>
+      <x:c r="I134" s="7"/>
     </x:row>
     <x:row r="135">
       <x:c r="G135" s="7"/>
+      <x:c r="I135" s="7"/>
     </x:row>
     <x:row r="136">
       <x:c r="G136" s="7"/>
+      <x:c r="I136" s="7"/>
     </x:row>
     <x:row r="137">
       <x:c r="G137" s="7"/>
+      <x:c r="I137" s="7"/>
     </x:row>
     <x:row r="138">
       <x:c r="G138" s="7"/>
+      <x:c r="I138" s="7"/>
     </x:row>
     <x:row r="139">
       <x:c r="G139" s="7"/>
+      <x:c r="I139" s="7"/>
     </x:row>
     <x:row r="140">
       <x:c r="G140" s="7"/>
+      <x:c r="I140" s="7"/>
     </x:row>
     <x:row r="141">
       <x:c r="G141" s="7"/>
+      <x:c r="I141" s="7"/>
     </x:row>
     <x:row r="142">
       <x:c r="G142" s="7"/>
+      <x:c r="I142" s="7"/>
     </x:row>
     <x:row r="143">
       <x:c r="G143" s="7"/>
+      <x:c r="I143" s="7"/>
     </x:row>
     <x:row r="144">
       <x:c r="G144" s="7"/>
+      <x:c r="I144" s="7"/>
     </x:row>
     <x:row r="145">
       <x:c r="G145" s="7"/>
+      <x:c r="I145" s="7"/>
     </x:row>
     <x:row r="146">
       <x:c r="G146" s="7"/>
+      <x:c r="I146" s="7"/>
     </x:row>
     <x:row r="147">
       <x:c r="G147" s="7"/>
+      <x:c r="I147" s="7"/>
     </x:row>
     <x:row r="148">
       <x:c r="G148" s="7"/>
+      <x:c r="I148" s="7"/>
     </x:row>
     <x:row r="149">
       <x:c r="G149" s="7"/>
+      <x:c r="I149" s="7"/>
     </x:row>
     <x:row r="150">
       <x:c r="G150" s="7"/>
+      <x:c r="I150" s="7"/>
     </x:row>
     <x:row r="151">
       <x:c r="G151" s="7"/>
+      <x:c r="I151" s="7"/>
     </x:row>
     <x:row r="152">
       <x:c r="G152" s="7"/>
+      <x:c r="I152" s="7"/>
     </x:row>
     <x:row r="153">
       <x:c r="G153" s="7"/>
+      <x:c r="I153" s="7"/>
     </x:row>
     <x:row r="154">
       <x:c r="G154" s="7"/>
+      <x:c r="I154" s="7"/>
     </x:row>
     <x:row r="155">
       <x:c r="G155" s="7"/>
+      <x:c r="I155" s="7"/>
     </x:row>
     <x:row r="156">
       <x:c r="G156" s="7"/>
+      <x:c r="I156" s="7"/>
     </x:row>
     <x:row r="157">
       <x:c r="G157" s="7"/>
+      <x:c r="I157" s="7"/>
     </x:row>
     <x:row r="158">
       <x:c r="G158" s="7"/>
+      <x:c r="I158" s="7"/>
     </x:row>
     <x:row r="159">
       <x:c r="G159" s="7"/>
+      <x:c r="I159" s="7"/>
     </x:row>
     <x:row r="160">
       <x:c r="G160" s="7"/>
+      <x:c r="I160" s="7"/>
     </x:row>
     <x:row r="161">
       <x:c r="G161" s="7"/>
+      <x:c r="I161" s="7"/>
     </x:row>
     <x:row r="162">
       <x:c r="G162" s="7"/>
+      <x:c r="I162" s="7"/>
     </x:row>
     <x:row r="163">
       <x:c r="G163" s="7"/>
+      <x:c r="I163" s="7"/>
     </x:row>
     <x:row r="164">
       <x:c r="G164" s="7"/>
+      <x:c r="I164" s="7"/>
     </x:row>
     <x:row r="165">
       <x:c r="G165" s="7"/>
+      <x:c r="I165" s="7"/>
     </x:row>
     <x:row r="166">
       <x:c r="G166" s="7"/>
+      <x:c r="I166" s="7"/>
     </x:row>
     <x:row r="167">
       <x:c r="G167" s="7"/>
+      <x:c r="I167" s="7"/>
     </x:row>
     <x:row r="168">
       <x:c r="G168" s="7"/>
+      <x:c r="I168" s="7"/>
     </x:row>
     <x:row r="169">
       <x:c r="G169" s="7"/>
+      <x:c r="I169" s="7"/>
     </x:row>
     <x:row r="170">
       <x:c r="G170" s="7"/>
+      <x:c r="I170" s="7"/>
     </x:row>
     <x:row r="171">
       <x:c r="G171" s="7"/>
+      <x:c r="I171" s="7"/>
     </x:row>
     <x:row r="172">
       <x:c r="G172" s="7"/>
+      <x:c r="I172" s="7"/>
     </x:row>
     <x:row r="173">
       <x:c r="G173" s="7"/>
+      <x:c r="I173" s="7"/>
     </x:row>
     <x:row r="174">
       <x:c r="G174" s="7"/>
+      <x:c r="I174" s="7"/>
     </x:row>
     <x:row r="175">
       <x:c r="G175" s="7"/>
+      <x:c r="I175" s="7"/>
     </x:row>
     <x:row r="176">
       <x:c r="G176" s="7"/>
+      <x:c r="I176" s="7"/>
     </x:row>
     <x:row r="177">
       <x:c r="G177" s="7"/>
+      <x:c r="I177" s="7"/>
     </x:row>
     <x:row r="178">
       <x:c r="G178" s="7"/>
+      <x:c r="I178" s="7"/>
     </x:row>
     <x:row r="179">
       <x:c r="G179" s="7"/>
+      <x:c r="I179" s="7"/>
     </x:row>
     <x:row r="180">
       <x:c r="G180" s="7"/>
+      <x:c r="I180" s="7"/>
     </x:row>
     <x:row r="181">
       <x:c r="G181" s="7"/>
+      <x:c r="I181" s="7"/>
     </x:row>
     <x:row r="182">
       <x:c r="G182" s="7"/>
+      <x:c r="I182" s="7"/>
     </x:row>
     <x:row r="183">
       <x:c r="G183" s="7"/>
+      <x:c r="I183" s="7"/>
     </x:row>
     <x:row r="184">
       <x:c r="G184" s="7"/>
+      <x:c r="I184" s="7"/>
     </x:row>
     <x:row r="185">
       <x:c r="G185" s="7"/>
+      <x:c r="I185" s="7"/>
     </x:row>
     <x:row r="186">
       <x:c r="G186" s="7"/>
+      <x:c r="I186" s="7"/>
     </x:row>
     <x:row r="187">
       <x:c r="G187" s="7"/>
+      <x:c r="I187" s="7"/>
     </x:row>
     <x:row r="188">
       <x:c r="G188" s="7"/>
+      <x:c r="I188" s="7"/>
     </x:row>
     <x:row r="189">
       <x:c r="G189" s="7"/>
+      <x:c r="I189" s="7"/>
     </x:row>
     <x:row r="190">
       <x:c r="G190" s="7"/>
+      <x:c r="I190" s="7"/>
     </x:row>
     <x:row r="191">
       <x:c r="G191" s="7"/>
+      <x:c r="I191" s="7"/>
     </x:row>
     <x:row r="192">
       <x:c r="G192" s="7"/>
+      <x:c r="I192" s="7"/>
     </x:row>
     <x:row r="193">
       <x:c r="G193" s="7"/>
+      <x:c r="I193" s="7"/>
     </x:row>
     <x:row r="194">
       <x:c r="G194" s="7"/>
+      <x:c r="I194" s="7"/>
     </x:row>
     <x:row r="195">
       <x:c r="G195" s="7"/>
+      <x:c r="I195" s="7"/>
     </x:row>
     <x:row r="196">
       <x:c r="G196" s="7"/>
+      <x:c r="I196" s="7"/>
     </x:row>
     <x:row r="197">
       <x:c r="G197" s="7"/>
+      <x:c r="I197" s="7"/>
     </x:row>
     <x:row r="198">
       <x:c r="G198" s="7"/>
+      <x:c r="I198" s="7"/>
     </x:row>
     <x:row r="199">
       <x:c r="G199" s="7"/>
+      <x:c r="I199" s="7"/>
     </x:row>
     <x:row r="200">
       <x:c r="G200" s="7"/>
+      <x:c r="I200" s="7"/>
     </x:row>
     <x:row r="201">
       <x:c r="G201" s="7"/>
+      <x:c r="I201" s="7"/>
     </x:row>
     <x:row r="202">
       <x:c r="G202" s="7"/>
+      <x:c r="I202" s="7"/>
     </x:row>
     <x:row r="203">
       <x:c r="G203" s="7"/>
+      <x:c r="I203" s="7"/>
     </x:row>
     <x:row r="204">
       <x:c r="G204" s="7"/>
+      <x:c r="I204" s="7"/>
     </x:row>
     <x:row r="205">
       <x:c r="G205" s="7"/>
+      <x:c r="I205" s="7"/>
     </x:row>
     <x:row r="206">
       <x:c r="G206" s="7"/>
+      <x:c r="I206" s="7"/>
     </x:row>
     <x:row r="207">
       <x:c r="G207" s="7"/>
+      <x:c r="I207" s="7"/>
     </x:row>
     <x:row r="208">
       <x:c r="G208" s="7"/>
+      <x:c r="I208" s="7"/>
     </x:row>
     <x:row r="209">
       <x:c r="G209" s="7"/>
+      <x:c r="I209" s="7"/>
     </x:row>
     <x:row r="210">
       <x:c r="G210" s="7"/>
+      <x:c r="I210" s="7"/>
     </x:row>
     <x:row r="211">
       <x:c r="G211" s="7"/>
+      <x:c r="I211" s="7"/>
     </x:row>
     <x:row r="212">
       <x:c r="G212" s="7"/>
+      <x:c r="I212" s="7"/>
     </x:row>
     <x:row r="213">
       <x:c r="G213" s="7"/>
+      <x:c r="I213" s="7"/>
     </x:row>
     <x:row r="214">
       <x:c r="G214" s="7"/>
+      <x:c r="I214" s="7"/>
     </x:row>
     <x:row r="215">
       <x:c r="G215" s="7"/>
+      <x:c r="I215" s="7"/>
     </x:row>
     <x:row r="216">
       <x:c r="G216" s="7"/>
+      <x:c r="I216" s="7"/>
     </x:row>
     <x:row r="217">
       <x:c r="G217" s="7"/>
+      <x:c r="I217" s="7"/>
     </x:row>
     <x:row r="218">
       <x:c r="G218" s="7"/>
+      <x:c r="I218" s="7"/>
     </x:row>
     <x:row r="219">
       <x:c r="G219" s="7"/>
+      <x:c r="I219" s="7"/>
     </x:row>
     <x:row r="220">
       <x:c r="G220" s="7"/>
+      <x:c r="I220" s="7"/>
     </x:row>
     <x:row r="221">
       <x:c r="G221" s="7"/>
+      <x:c r="I221" s="7"/>
     </x:row>
     <x:row r="222">
       <x:c r="G222" s="7"/>
+      <x:c r="I222" s="7"/>
     </x:row>
     <x:row r="223">
       <x:c r="G223" s="7"/>
+      <x:c r="I223" s="7"/>
     </x:row>
     <x:row r="224">
       <x:c r="G224" s="7"/>
+      <x:c r="I224" s="7"/>
     </x:row>
     <x:row r="225">
       <x:c r="G225" s="7"/>
+      <x:c r="I225" s="7"/>
     </x:row>
     <x:row r="226">
       <x:c r="G226" s="7"/>
+      <x:c r="I226" s="7"/>
     </x:row>
     <x:row r="227">
       <x:c r="G227" s="7"/>
+      <x:c r="I227" s="7"/>
     </x:row>
     <x:row r="228">
       <x:c r="G228" s="7"/>
+      <x:c r="I228" s="7"/>
     </x:row>
     <x:row r="229">
       <x:c r="G229" s="7"/>
+      <x:c r="I229" s="7"/>
     </x:row>
     <x:row r="230">
       <x:c r="G230" s="7"/>
+      <x:c r="I230" s="7"/>
     </x:row>
     <x:row r="231">
       <x:c r="G231" s="7"/>
+      <x:c r="I231" s="7"/>
     </x:row>
     <x:row r="232">
       <x:c r="G232" s="7"/>
+      <x:c r="I232" s="7"/>
     </x:row>
     <x:row r="233">
       <x:c r="G233" s="7"/>
+      <x:c r="I233" s="7"/>
     </x:row>
     <x:row r="234">
       <x:c r="G234" s="7"/>
+      <x:c r="I234" s="7"/>
     </x:row>
     <x:row r="235">
       <x:c r="G235" s="7"/>
+      <x:c r="I235" s="7"/>
     </x:row>
     <x:row r="236">
       <x:c r="G236" s="7"/>
+      <x:c r="I236" s="7"/>
     </x:row>
     <x:row r="237">
       <x:c r="G237" s="7"/>
+      <x:c r="I237" s="7"/>
     </x:row>
     <x:row r="238">
       <x:c r="G238" s="7"/>
+      <x:c r="I238" s="7"/>
     </x:row>
     <x:row r="239">
       <x:c r="G239" s="7"/>
+      <x:c r="I239" s="7"/>
     </x:row>
     <x:row r="240">
       <x:c r="G240" s="7"/>
+      <x:c r="I240" s="7"/>
     </x:row>
     <x:row r="241">
       <x:c r="G241" s="7"/>
+      <x:c r="I241" s="7"/>
     </x:row>
     <x:row r="242">
       <x:c r="G242" s="7"/>
+      <x:c r="I242" s="7"/>
     </x:row>
     <x:row r="243">
       <x:c r="G243" s="7"/>
+      <x:c r="I243" s="7"/>
     </x:row>
     <x:row r="244">
       <x:c r="G244" s="7"/>
+      <x:c r="I244" s="7"/>
     </x:row>
     <x:row r="245">
       <x:c r="G245" s="7"/>
+      <x:c r="I245" s="7"/>
     </x:row>
     <x:row r="246">
       <x:c r="G246" s="7"/>
+      <x:c r="I246" s="7"/>
     </x:row>
     <x:row r="247">
       <x:c r="G247" s="7"/>
+      <x:c r="I247" s="7"/>
     </x:row>
     <x:row r="248">
       <x:c r="G248" s="7"/>
+      <x:c r="I248" s="7"/>
     </x:row>
     <x:row r="249">
       <x:c r="G249" s="7"/>
+      <x:c r="I249" s="7"/>
     </x:row>
     <x:row r="250">
       <x:c r="G250" s="7"/>
+      <x:c r="I250" s="7"/>
     </x:row>
     <x:row r="251">
       <x:c r="G251" s="7"/>
+      <x:c r="I251" s="7"/>
     </x:row>
     <x:row r="252">
       <x:c r="G252" s="7"/>
+      <x:c r="I252" s="7"/>
     </x:row>
     <x:row r="253">
       <x:c r="G253" s="7"/>
+      <x:c r="I253" s="7"/>
     </x:row>
     <x:row r="254">
       <x:c r="G254" s="7"/>
+      <x:c r="I254" s="7"/>
     </x:row>
     <x:row r="255">
       <x:c r="G255" s="7"/>
+      <x:c r="I255" s="7"/>
     </x:row>
     <x:row r="256">
       <x:c r="G256" s="7"/>
+      <x:c r="I256" s="7"/>
     </x:row>
     <x:row r="257">
       <x:c r="G257" s="7"/>
+      <x:c r="I257" s="7"/>
     </x:row>
     <x:row r="258">
       <x:c r="G258" s="7"/>
+      <x:c r="I258" s="7"/>
     </x:row>
     <x:row r="259">
       <x:c r="G259" s="7"/>
+      <x:c r="I259" s="7"/>
     </x:row>
     <x:row r="260">
       <x:c r="G260" s="7"/>
+      <x:c r="I260" s="7"/>
     </x:row>
     <x:row r="261">
       <x:c r="G261" s="7"/>
+      <x:c r="I261" s="7"/>
     </x:row>
     <x:row r="262">
       <x:c r="G262" s="7"/>
+      <x:c r="I262" s="7"/>
     </x:row>
     <x:row r="263">
       <x:c r="G263" s="7"/>
+      <x:c r="I263" s="7"/>
     </x:row>
     <x:row r="264">
       <x:c r="G264" s="7"/>
+      <x:c r="I264" s="7"/>
     </x:row>
     <x:row r="265">
       <x:c r="G265" s="7"/>
+      <x:c r="I265" s="7"/>
     </x:row>
     <x:row r="266">
       <x:c r="G266" s="7"/>
+      <x:c r="I266" s="7"/>
     </x:row>
     <x:row r="267">
       <x:c r="G267" s="7"/>
+      <x:c r="I267" s="7"/>
     </x:row>
     <x:row r="268">
       <x:c r="G268" s="7"/>
+      <x:c r="I268" s="7"/>
     </x:row>
     <x:row r="269">
       <x:c r="G269" s="7"/>
+      <x:c r="I269" s="7"/>
     </x:row>
     <x:row r="270">
       <x:c r="G270" s="7"/>
+      <x:c r="I270" s="7"/>
     </x:row>
     <x:row r="271">
       <x:c r="G271" s="7"/>
+      <x:c r="I271" s="7"/>
     </x:row>
     <x:row r="272">
       <x:c r="G272" s="7"/>
+      <x:c r="I272" s="7"/>
     </x:row>
     <x:row r="273">
       <x:c r="G273" s="7"/>
+      <x:c r="I273" s="7"/>
     </x:row>
     <x:row r="274">
       <x:c r="G274" s="7"/>
+      <x:c r="I274" s="7"/>
     </x:row>
     <x:row r="275">
       <x:c r="G275" s="7"/>
+      <x:c r="I275" s="7"/>
     </x:row>
     <x:row r="276">
       <x:c r="G276" s="7"/>
+      <x:c r="I276" s="7"/>
     </x:row>
     <x:row r="277">
       <x:c r="G277" s="7"/>
+      <x:c r="I277" s="7"/>
     </x:row>
     <x:row r="278">
       <x:c r="G278" s="7"/>
+      <x:c r="I278" s="7"/>
     </x:row>
     <x:row r="279">
       <x:c r="G279" s="7"/>
+      <x:c r="I279" s="7"/>
     </x:row>
     <x:row r="280">
       <x:c r="G280" s="7"/>
+      <x:c r="I280" s="7"/>
     </x:row>
     <x:row r="281">
       <x:c r="G281" s="7"/>
+      <x:c r="I281" s="7"/>
     </x:row>
     <x:row r="282">
       <x:c r="G282" s="7"/>
+      <x:c r="I282" s="7"/>
     </x:row>
     <x:row r="283">
       <x:c r="G283" s="7"/>
+      <x:c r="I283" s="7"/>
     </x:row>
     <x:row r="284">
       <x:c r="G284" s="7"/>
+      <x:c r="I284" s="7"/>
     </x:row>
     <x:row r="285">
       <x:c r="G285" s="7"/>
+      <x:c r="I285" s="7"/>
     </x:row>
     <x:row r="286">
       <x:c r="G286" s="7"/>
+      <x:c r="I286" s="7"/>
     </x:row>
     <x:row r="287">
       <x:c r="G287" s="7"/>
+      <x:c r="I287" s="7"/>
     </x:row>
     <x:row r="288">
       <x:c r="G288" s="7"/>
+      <x:c r="I288" s="7"/>
     </x:row>
     <x:row r="289">
       <x:c r="G289" s="7"/>
+      <x:c r="I289" s="7"/>
     </x:row>
     <x:row r="290">
       <x:c r="G290" s="7"/>
+      <x:c r="I290" s="7"/>
     </x:row>
     <x:row r="291">
       <x:c r="G291" s="7"/>
+      <x:c r="I291" s="7"/>
     </x:row>
     <x:row r="292">
       <x:c r="G292" s="7"/>
+      <x:c r="I292" s="7"/>
     </x:row>
     <x:row r="293">
       <x:c r="G293" s="7"/>
+      <x:c r="I293" s="7"/>
     </x:row>
     <x:row r="294">
       <x:c r="G294" s="7"/>
+      <x:c r="I294" s="7"/>
     </x:row>
     <x:row r="295">
       <x:c r="G295" s="7"/>
+      <x:c r="I295" s="7"/>
     </x:row>
     <x:row r="296">
       <x:c r="G296" s="7"/>
+      <x:c r="I296" s="7"/>
     </x:row>
     <x:row r="297">
       <x:c r="G297" s="7"/>
+      <x:c r="I297" s="7"/>
     </x:row>
     <x:row r="298">
       <x:c r="G298" s="7"/>
+      <x:c r="I298" s="7"/>
     </x:row>
     <x:row r="299">
       <x:c r="G299" s="7"/>
+      <x:c r="I299" s="7"/>
     </x:row>
     <x:row r="300">
       <x:c r="G300" s="7"/>
+      <x:c r="I300" s="7"/>
     </x:row>
     <x:row r="301">
       <x:c r="G301" s="7"/>
+      <x:c r="I301" s="7"/>
     </x:row>
     <x:row r="302">
       <x:c r="G302" s="7"/>
+      <x:c r="I302" s="7"/>
     </x:row>
     <x:row r="303">
       <x:c r="G303" s="7"/>
+      <x:c r="I303" s="7"/>
     </x:row>
     <x:row r="304">
       <x:c r="G304" s="7"/>
+      <x:c r="I304" s="7"/>
     </x:row>
     <x:row r="305">
       <x:c r="G305" s="7"/>
+      <x:c r="I305" s="7"/>
     </x:row>
     <x:row r="306">
       <x:c r="G306" s="7"/>
+      <x:c r="I306" s="7"/>
     </x:row>
     <x:row r="307">
       <x:c r="G307" s="7"/>
+      <x:c r="I307" s="7"/>
     </x:row>
     <x:row r="308">
       <x:c r="G308" s="7"/>
+      <x:c r="I308" s="7"/>
     </x:row>
     <x:row r="309">
       <x:c r="G309" s="7"/>
+      <x:c r="I309" s="7"/>
     </x:row>
     <x:row r="310">
       <x:c r="G310" s="7"/>
+      <x:c r="I310" s="7"/>
     </x:row>
     <x:row r="311">
       <x:c r="G311" s="7"/>
+      <x:c r="I311" s="7"/>
     </x:row>
     <x:row r="312">
       <x:c r="G312" s="7"/>
+      <x:c r="I312" s="7"/>
     </x:row>
     <x:row r="313">
       <x:c r="G313" s="7"/>
+      <x:c r="I313" s="7"/>
     </x:row>
     <x:row r="314">
       <x:c r="G314" s="7"/>
+      <x:c r="I314" s="7"/>
     </x:row>
     <x:row r="315">
       <x:c r="G315" s="7"/>
+      <x:c r="I315" s="7"/>
     </x:row>
     <x:row r="316">
       <x:c r="G316" s="7"/>
+      <x:c r="I316" s="7"/>
     </x:row>
     <x:row r="317">
       <x:c r="G317" s="7"/>
+      <x:c r="I317" s="7"/>
     </x:row>
     <x:row r="318">
       <x:c r="G318" s="7"/>
+      <x:c r="I318" s="7"/>
     </x:row>
     <x:row r="319">
       <x:c r="G319" s="7"/>
+      <x:c r="I319" s="7"/>
     </x:row>
     <x:row r="320">
       <x:c r="G320" s="7"/>
+      <x:c r="I320" s="7"/>
     </x:row>
     <x:row r="321">
       <x:c r="G321" s="7"/>
+      <x:c r="I321" s="7"/>
     </x:row>
     <x:row r="322">
       <x:c r="G322" s="7"/>
+      <x:c r="I322" s="7"/>
     </x:row>
     <x:row r="323">
       <x:c r="G323" s="7"/>
+      <x:c r="I323" s="7"/>
     </x:row>
     <x:row r="324">
       <x:c r="G324" s="7"/>
+      <x:c r="I324" s="7"/>
     </x:row>
     <x:row r="325">
       <x:c r="G325" s="7"/>
+      <x:c r="I325" s="7"/>
     </x:row>
     <x:row r="326">
       <x:c r="G326" s="7"/>
+      <x:c r="I326" s="7"/>
     </x:row>
     <x:row r="327">
       <x:c r="G327" s="7"/>
+      <x:c r="I327" s="7"/>
     </x:row>
     <x:row r="328">
       <x:c r="G328" s="7"/>
+      <x:c r="I328" s="7"/>
     </x:row>
     <x:row r="329">
       <x:c r="G329" s="7"/>
+      <x:c r="I329" s="7"/>
     </x:row>
     <x:row r="330">
       <x:c r="G330" s="7"/>
+      <x:c r="I330" s="7"/>
     </x:row>
     <x:row r="331">
       <x:c r="G331" s="7"/>
+      <x:c r="I331" s="7"/>
     </x:row>
     <x:row r="332">
       <x:c r="G332" s="7"/>
+      <x:c r="I332" s="7"/>
     </x:row>
     <x:row r="333">
       <x:c r="G333" s="7"/>
+      <x:c r="I333" s="7"/>
     </x:row>
     <x:row r="334">
       <x:c r="G334" s="7"/>
+      <x:c r="I334" s="7"/>
     </x:row>
     <x:row r="335">
       <x:c r="G335" s="7"/>
+      <x:c r="I335" s="7"/>
     </x:row>
     <x:row r="336">
       <x:c r="G336" s="7"/>
+      <x:c r="I336" s="7"/>
     </x:row>
     <x:row r="337">
       <x:c r="G337" s="7"/>
+      <x:c r="I337" s="7"/>
     </x:row>
     <x:row r="338">
       <x:c r="G338" s="7"/>
+      <x:c r="I338" s="7"/>
     </x:row>
     <x:row r="339">
       <x:c r="G339" s="7"/>
+      <x:c r="I339" s="7"/>
     </x:row>
     <x:row r="340">
       <x:c r="G340" s="7"/>
+      <x:c r="I340" s="7"/>
     </x:row>
     <x:row r="341">
       <x:c r="G341" s="7"/>
+      <x:c r="I341" s="7"/>
     </x:row>
     <x:row r="342">
       <x:c r="G342" s="7"/>
+      <x:c r="I342" s="7"/>
     </x:row>
     <x:row r="343">
       <x:c r="G343" s="7"/>
+      <x:c r="I343" s="7"/>
     </x:row>
     <x:row r="344">
       <x:c r="G344" s="7"/>
+      <x:c r="I344" s="7"/>
     </x:row>
     <x:row r="345">
       <x:c r="G345" s="7"/>
+      <x:c r="I345" s="7"/>
     </x:row>
     <x:row r="346">
       <x:c r="G346" s="7"/>
+      <x:c r="I346" s="7"/>
     </x:row>
     <x:row r="347">
       <x:c r="G347" s="7"/>
+      <x:c r="I347" s="7"/>
     </x:row>
     <x:row r="348">
       <x:c r="G348" s="7"/>
+      <x:c r="I348" s="7"/>
     </x:row>
     <x:row r="349">
       <x:c r="G349" s="7"/>
+      <x:c r="I349" s="7"/>
     </x:row>
     <x:row r="350">
       <x:c r="G350" s="7"/>
+      <x:c r="I350" s="7"/>
     </x:row>
     <x:row r="351">
       <x:c r="G351" s="7"/>
+      <x:c r="I351" s="7"/>
     </x:row>
     <x:row r="352">
       <x:c r="G352" s="7"/>
+      <x:c r="I352" s="7"/>
     </x:row>
     <x:row r="353">
       <x:c r="G353" s="7"/>
+      <x:c r="I353" s="7"/>
     </x:row>
     <x:row r="354">
       <x:c r="G354" s="7"/>
+      <x:c r="I354" s="7"/>
     </x:row>
     <x:row r="355">
       <x:c r="G355" s="7"/>
+      <x:c r="I355" s="7"/>
     </x:row>
     <x:row r="356">
       <x:c r="G356" s="7"/>
+      <x:c r="I356" s="7"/>
     </x:row>
     <x:row r="357">
       <x:c r="G357" s="7"/>
+      <x:c r="I357" s="7"/>
     </x:row>
     <x:row r="358">
       <x:c r="G358" s="7"/>
+      <x:c r="I358" s="7"/>
     </x:row>
     <x:row r="359">
       <x:c r="G359" s="7"/>
+      <x:c r="I359" s="7"/>
     </x:row>
     <x:row r="360">
       <x:c r="G360" s="7"/>
+      <x:c r="I360" s="7"/>
     </x:row>
     <x:row r="361">
       <x:c r="G361" s="7"/>
+      <x:c r="I361" s="7"/>
     </x:row>
     <x:row r="362">
       <x:c r="G362" s="7"/>
+      <x:c r="I362" s="7"/>
     </x:row>
     <x:row r="363">
       <x:c r="G363" s="7"/>
+      <x:c r="I363" s="7"/>
     </x:row>
     <x:row r="364">
       <x:c r="G364" s="7"/>
+      <x:c r="I364" s="7"/>
     </x:row>
     <x:row r="365">
       <x:c r="G365" s="7"/>
+      <x:c r="I365" s="7"/>
     </x:row>
     <x:row r="366">
       <x:c r="G366" s="7"/>
+      <x:c r="I366" s="7"/>
     </x:row>
     <x:row r="367">
       <x:c r="G367" s="7"/>
+      <x:c r="I367" s="7"/>
     </x:row>
     <x:row r="368">
       <x:c r="G368" s="7"/>
+      <x:c r="I368" s="7"/>
     </x:row>
     <x:row r="369">
       <x:c r="G369" s="7"/>
+      <x:c r="I369" s="7"/>
     </x:row>
     <x:row r="370">
       <x:c r="G370" s="7"/>
+      <x:c r="I370" s="7"/>
     </x:row>
     <x:row r="371">
       <x:c r="G371" s="7"/>
+      <x:c r="I371" s="7"/>
     </x:row>
     <x:row r="372">
       <x:c r="G372" s="7"/>
+      <x:c r="I372" s="7"/>
     </x:row>
     <x:row r="373">
       <x:c r="G373" s="7"/>
+      <x:c r="I373" s="7"/>
     </x:row>
     <x:row r="374">
       <x:c r="G374" s="7"/>
+      <x:c r="I374" s="7"/>
     </x:row>
     <x:row r="375">
       <x:c r="G375" s="7"/>
+      <x:c r="I375" s="7"/>
     </x:row>
     <x:row r="376">
       <x:c r="G376" s="7"/>
+      <x:c r="I376" s="7"/>
     </x:row>
     <x:row r="377">
       <x:c r="G377" s="7"/>
+      <x:c r="I377" s="7"/>
     </x:row>
     <x:row r="378">
       <x:c r="G378" s="7"/>
+      <x:c r="I378" s="7"/>
     </x:row>
     <x:row r="379">
       <x:c r="G379" s="7"/>
+      <x:c r="I379" s="7"/>
     </x:row>
     <x:row r="380">
       <x:c r="G380" s="7"/>
+      <x:c r="I380" s="7"/>
     </x:row>
     <x:row r="381">
       <x:c r="G381" s="7"/>
+      <x:c r="I381" s="7"/>
     </x:row>
     <x:row r="382">
       <x:c r="G382" s="7"/>
+      <x:c r="I382" s="7"/>
     </x:row>
     <x:row r="383">
       <x:c r="G383" s="7"/>
+      <x:c r="I383" s="7"/>
     </x:row>
     <x:row r="384">
       <x:c r="G384" s="7"/>
+      <x:c r="I384" s="7"/>
     </x:row>
     <x:row r="385">
       <x:c r="G385" s="7"/>
+      <x:c r="I385" s="7"/>
     </x:row>
     <x:row r="386">
       <x:c r="G386" s="7"/>
+      <x:c r="I386" s="7"/>
     </x:row>
     <x:row r="387">
       <x:c r="G387" s="7"/>
+      <x:c r="I387" s="7"/>
     </x:row>
     <x:row r="388">
       <x:c r="G388" s="7"/>
+      <x:c r="I388" s="7"/>
     </x:row>
     <x:row r="389">
       <x:c r="G389" s="7"/>
+      <x:c r="I389" s="7"/>
     </x:row>
     <x:row r="390">
       <x:c r="G390" s="7"/>
+      <x:c r="I390" s="7"/>
     </x:row>
     <x:row r="391">
       <x:c r="G391" s="7"/>
+      <x:c r="I391" s="7"/>
     </x:row>
     <x:row r="392">
       <x:c r="G392" s="7"/>
+      <x:c r="I392" s="7"/>
     </x:row>
     <x:row r="393">
       <x:c r="G393" s="7"/>
+      <x:c r="I393" s="7"/>
     </x:row>
     <x:row r="394">
       <x:c r="G394" s="7"/>
+      <x:c r="I394" s="7"/>
     </x:row>
     <x:row r="395">
       <x:c r="G395" s="7"/>
+      <x:c r="I395" s="7"/>
     </x:row>
     <x:row r="396">
       <x:c r="G396" s="7"/>
+      <x:c r="I396" s="7"/>
     </x:row>
     <x:row r="397">
       <x:c r="G397" s="7"/>
+      <x:c r="I397" s="7"/>
     </x:row>
     <x:row r="398">
       <x:c r="G398" s="7"/>
+      <x:c r="I398" s="7"/>
     </x:row>
     <x:row r="399">
       <x:c r="G399" s="7"/>
+      <x:c r="I399" s="7"/>
     </x:row>
     <x:row r="400">
       <x:c r="G400" s="7"/>
+      <x:c r="I400" s="7"/>
     </x:row>
     <x:row r="401">
       <x:c r="G401" s="7"/>
+      <x:c r="I401" s="7"/>
     </x:row>
     <x:row r="402">
       <x:c r="G402" s="7"/>
+      <x:c r="I402" s="7"/>
     </x:row>
     <x:row r="403">
       <x:c r="G403" s="7"/>
+      <x:c r="I403" s="7"/>
     </x:row>
     <x:row r="404">
       <x:c r="G404" s="7"/>
+      <x:c r="I404" s="7"/>
     </x:row>
     <x:row r="405">
       <x:c r="G405" s="7"/>
+      <x:c r="I405" s="7"/>
     </x:row>
     <x:row r="406">
       <x:c r="G406" s="7"/>
+      <x:c r="I406" s="7"/>
     </x:row>
     <x:row r="407">
       <x:c r="G407" s="7"/>
+      <x:c r="I407" s="7"/>
     </x:row>
     <x:row r="408">
       <x:c r="G408" s="7"/>
+      <x:c r="I408" s="7"/>
     </x:row>
     <x:row r="409">
       <x:c r="G409" s="7"/>
+      <x:c r="I409" s="7"/>
     </x:row>
     <x:row r="410">
       <x:c r="G410" s="7"/>
+      <x:c r="I410" s="7"/>
     </x:row>
     <x:row r="411">
       <x:c r="G411" s="7"/>
+      <x:c r="I411" s="7"/>
     </x:row>
     <x:row r="412">
       <x:c r="G412" s="7"/>
+      <x:c r="I412" s="7"/>
     </x:row>
     <x:row r="413">
       <x:c r="G413" s="7"/>
+      <x:c r="I413" s="7"/>
     </x:row>
     <x:row r="414">
       <x:c r="G414" s="7"/>
+      <x:c r="I414" s="7"/>
     </x:row>
     <x:row r="415">
       <x:c r="G415" s="7"/>
+      <x:c r="I415" s="7"/>
     </x:row>
     <x:row r="416">
       <x:c r="G416" s="7"/>
+      <x:c r="I416" s="7"/>
     </x:row>
     <x:row r="417">
       <x:c r="G417" s="7"/>
+      <x:c r="I417" s="7"/>
     </x:row>
     <x:row r="418">
       <x:c r="G418" s="7"/>
+      <x:c r="I418" s="7"/>
     </x:row>
     <x:row r="419">
       <x:c r="G419" s="7"/>
+      <x:c r="I419" s="7"/>
     </x:row>
     <x:row r="420">
       <x:c r="G420" s="7"/>
+      <x:c r="I420" s="7"/>
     </x:row>
     <x:row r="421">
       <x:c r="G421" s="7"/>
+      <x:c r="I421" s="7"/>
     </x:row>
     <x:row r="422">
       <x:c r="G422" s="7"/>
+      <x:c r="I422" s="7"/>
     </x:row>
     <x:row r="423">
       <x:c r="G423" s="7"/>
+      <x:c r="I423" s="7"/>
     </x:row>
     <x:row r="424">
       <x:c r="G424" s="7"/>
+      <x:c r="I424" s="7"/>
     </x:row>
     <x:row r="425">
       <x:c r="G425" s="7"/>
+      <x:c r="I425" s="7"/>
     </x:row>
     <x:row r="426">
       <x:c r="G426" s="7"/>
+      <x:c r="I426" s="7"/>
     </x:row>
     <x:row r="427">
       <x:c r="G427" s="7"/>
+      <x:c r="I427" s="7"/>
     </x:row>
     <x:row r="428">
       <x:c r="G428" s="7"/>
+      <x:c r="I428" s="7"/>
     </x:row>
     <x:row r="429">
       <x:c r="G429" s="7"/>
+      <x:c r="I429" s="7"/>
     </x:row>
     <x:row r="430">
       <x:c r="G430" s="7"/>
+      <x:c r="I430" s="7"/>
     </x:row>
     <x:row r="431">
       <x:c r="G431" s="7"/>
+      <x:c r="I431" s="7"/>
     </x:row>
     <x:row r="432">
       <x:c r="G432" s="7"/>
+      <x:c r="I432" s="7"/>
     </x:row>
     <x:row r="433">
       <x:c r="G433" s="7"/>
+      <x:c r="I433" s="7"/>
     </x:row>
     <x:row r="434">
       <x:c r="G434" s="7"/>
+      <x:c r="I434" s="7"/>
     </x:row>
     <x:row r="435">
       <x:c r="G435" s="7"/>
+      <x:c r="I435" s="7"/>
     </x:row>
     <x:row r="436">
       <x:c r="G436" s="7"/>
+      <x:c r="I436" s="7"/>
     </x:row>
     <x:row r="437">
       <x:c r="G437" s="7"/>
+      <x:c r="I437" s="7"/>
     </x:row>
     <x:row r="438">
       <x:c r="G438" s="7"/>
+      <x:c r="I438" s="7"/>
     </x:row>
     <x:row r="439">
       <x:c r="G439" s="7"/>
+      <x:c r="I439" s="7"/>
     </x:row>
     <x:row r="440">
       <x:c r="G440" s="7"/>
+      <x:c r="I440" s="7"/>
     </x:row>
     <x:row r="441">
       <x:c r="G441" s="7"/>
+      <x:c r="I441" s="7"/>
     </x:row>
     <x:row r="442">
       <x:c r="G442" s="7"/>
+      <x:c r="I442" s="7"/>
     </x:row>
     <x:row r="443">
       <x:c r="G443" s="7"/>
+      <x:c r="I443" s="7"/>
     </x:row>
     <x:row r="444">
       <x:c r="G444" s="7"/>
+      <x:c r="I444" s="7"/>
     </x:row>
     <x:row r="445">
       <x:c r="G445" s="7"/>
+      <x:c r="I445" s="7"/>
     </x:row>
     <x:row r="446">
       <x:c r="G446" s="7"/>
+      <x:c r="I446" s="7"/>
     </x:row>
     <x:row r="447">
       <x:c r="G447" s="7"/>
+      <x:c r="I447" s="7"/>
     </x:row>
     <x:row r="448">
       <x:c r="G448" s="7"/>
+      <x:c r="I448" s="7"/>
     </x:row>
     <x:row r="449">
       <x:c r="G449" s="7"/>
+      <x:c r="I449" s="7"/>
     </x:row>
     <x:row r="450">
       <x:c r="G450" s="7"/>
+      <x:c r="I450" s="7"/>
     </x:row>
     <x:row r="451">
       <x:c r="G451" s="7"/>
+      <x:c r="I451" s="7"/>
     </x:row>
     <x:row r="452">
       <x:c r="G452" s="7"/>
+      <x:c r="I452" s="7"/>
     </x:row>
     <x:row r="453">
       <x:c r="G453" s="7"/>
+      <x:c r="I453" s="7"/>
     </x:row>
     <x:row r="454">
       <x:c r="G454" s="7"/>
+      <x:c r="I454" s="7"/>
     </x:row>
     <x:row r="455">
       <x:c r="G455" s="7"/>
+      <x:c r="I455" s="7"/>
     </x:row>
     <x:row r="456">
       <x:c r="G456" s="7"/>
+      <x:c r="I456" s="7"/>
     </x:row>
     <x:row r="457">
       <x:c r="G457" s="7"/>
+      <x:c r="I457" s="7"/>
     </x:row>
     <x:row r="458">
       <x:c r="G458" s="7"/>
+      <x:c r="I458" s="7"/>
     </x:row>
     <x:row r="459">
       <x:c r="G459" s="7"/>
+      <x:c r="I459" s="7"/>
     </x:row>
     <x:row r="460">
       <x:c r="G460" s="7"/>
+      <x:c r="I460" s="7"/>
     </x:row>
     <x:row r="461">
       <x:c r="G461" s="7"/>
+      <x:c r="I461" s="7"/>
     </x:row>
     <x:row r="462">
       <x:c r="G462" s="7"/>
+      <x:c r="I462" s="7"/>
     </x:row>
     <x:row r="463">
       <x:c r="G463" s="7"/>
+      <x:c r="I463" s="7"/>
     </x:row>
     <x:row r="464">
       <x:c r="G464" s="7"/>
+      <x:c r="I464" s="7"/>
     </x:row>
     <x:row r="465">
       <x:c r="G465" s="7"/>
+      <x:c r="I465" s="7"/>
     </x:row>
     <x:row r="466">
       <x:c r="G466" s="7"/>
+      <x:c r="I466" s="7"/>
     </x:row>
     <x:row r="467">
       <x:c r="G467" s="7"/>
+      <x:c r="I467" s="7"/>
     </x:row>
     <x:row r="468">
       <x:c r="G468" s="7"/>
+      <x:c r="I468" s="7"/>
     </x:row>
     <x:row r="469">
       <x:c r="G469" s="7"/>
+      <x:c r="I469" s="7"/>
     </x:row>
     <x:row r="470">
       <x:c r="G470" s="7"/>
+      <x:c r="I470" s="7"/>
     </x:row>
     <x:row r="471">
       <x:c r="G471" s="7"/>
+      <x:c r="I471" s="7"/>
     </x:row>
     <x:row r="472">
       <x:c r="G472" s="7"/>
+      <x:c r="I472" s="7"/>
     </x:row>
     <x:row r="473">
       <x:c r="G473" s="7"/>
+      <x:c r="I473" s="7"/>
     </x:row>
     <x:row r="474">
       <x:c r="G474" s="7"/>
+      <x:c r="I474" s="7"/>
     </x:row>
     <x:row r="475">
       <x:c r="G475" s="7"/>
+      <x:c r="I475" s="7"/>
     </x:row>
     <x:row r="476">
       <x:c r="G476" s="7"/>
+      <x:c r="I476" s="7"/>
     </x:row>
     <x:row r="477">
       <x:c r="G477" s="7"/>
+      <x:c r="I477" s="7"/>
     </x:row>
     <x:row r="478">
       <x:c r="G478" s="7"/>
+      <x:c r="I478" s="7"/>
     </x:row>
     <x:row r="479">
       <x:c r="G479" s="7"/>
+      <x:c r="I479" s="7"/>
     </x:row>
     <x:row r="480">
       <x:c r="G480" s="7"/>
+      <x:c r="I480" s="7"/>
     </x:row>
     <x:row r="481">
       <x:c r="G481" s="7"/>
+      <x:c r="I481" s="7"/>
     </x:row>
     <x:row r="482">
       <x:c r="G482" s="7"/>
+      <x:c r="I482" s="7"/>
     </x:row>
     <x:row r="483">
       <x:c r="G483" s="7"/>
+      <x:c r="I483" s="7"/>
     </x:row>
     <x:row r="484">
       <x:c r="G484" s="7"/>
+      <x:c r="I484" s="7"/>
     </x:row>
     <x:row r="485">
       <x:c r="G485" s="7"/>
+      <x:c r="I485" s="7"/>
     </x:row>
     <x:row r="486">
       <x:c r="G486" s="7"/>
+      <x:c r="I486" s="7"/>
     </x:row>
     <x:row r="487">
       <x:c r="G487" s="7"/>
+      <x:c r="I487" s="7"/>
     </x:row>
     <x:row r="488">
       <x:c r="G488" s="7"/>
+      <x:c r="I488" s="7"/>
     </x:row>
     <x:row r="489">
       <x:c r="G489" s="7"/>
+      <x:c r="I489" s="7"/>
     </x:row>
     <x:row r="490">
       <x:c r="G490" s="7"/>
+      <x:c r="I490" s="7"/>
     </x:row>
     <x:row r="491">
       <x:c r="G491" s="7"/>
+      <x:c r="I491" s="7"/>
     </x:row>
     <x:row r="492">
       <x:c r="G492" s="7"/>
+      <x:c r="I492" s="7"/>
     </x:row>
     <x:row r="493">
       <x:c r="G493" s="7"/>
+      <x:c r="I493" s="7"/>
     </x:row>
     <x:row r="494">
       <x:c r="G494" s="7"/>
+      <x:c r="I494" s="7"/>
     </x:row>
     <x:row r="495">
       <x:c r="G495" s="7"/>
+      <x:c r="I495" s="7"/>
     </x:row>
     <x:row r="496">
       <x:c r="G496" s="7"/>
+      <x:c r="I496" s="7"/>
     </x:row>
     <x:row r="497">
       <x:c r="G497" s="7"/>
+      <x:c r="I497" s="7"/>
     </x:row>
     <x:row r="498">
       <x:c r="G498" s="7"/>
+      <x:c r="I498" s="7"/>
     </x:row>
     <x:row r="499">
       <x:c r="G499" s="7"/>
+      <x:c r="I499" s="7"/>
     </x:row>
     <x:row r="500">
       <x:c r="G500" s="7"/>
+      <x:c r="I500" s="7"/>
     </x:row>
     <x:row r="501">
       <x:c r="G501" s="7"/>
+      <x:c r="I501" s="7"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">

</xml_diff>